<commit_message>
Network map: add China domestic line across A-E (94 people); stage coverage batches
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012LRydPx3p71npFqtrfS6Ef
</commit_message>
<xml_diff>
--- a/iLands_Agent_Economy_Network_2026-07-01.xlsx
+++ b/iLands_Agent_Economy_Network_2026-07-01.xlsx
@@ -11,7 +11,7 @@
     <sheet name="How to use" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Agent Economy Network'!$A$4:$J$80</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Agent Economy Network'!$A$4:$J$98</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -613,7 +613,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J80"/>
+  <dimension ref="A1:J98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4646,8 +4646,944 @@
         </is>
       </c>
     </row>
+    <row r="81">
+      <c r="A81" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B81" s="5" t="inlineStr">
+        <is>
+          <t>A. Framework &amp; Infra Builders</t>
+        </is>
+      </c>
+      <c r="C81" s="6" t="inlineStr">
+        <is>
+          <t>Wu Chenglin (吴承霖)</t>
+        </is>
+      </c>
+      <c r="D81" s="5" t="inlineStr">
+        <is>
+          <t>DeepWisdom (深度赋智) — MetaGPT founder</t>
+        </is>
+      </c>
+      <c r="E81" s="5" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="F81" s="5" t="inlineStr">
+        <is>
+          <t>MetaGPT = top OSS multi-agent framework ('a software company of agents'); huge global stars</t>
+        </is>
+      </c>
+      <c r="G81" s="5" t="inlineStr">
+        <is>
+          <t>Multi-agent society (roles collaborate) directly parallels iLands residents — CN builder anchor</t>
+        </is>
+      </c>
+      <c r="H81" s="5" t="inlineStr">
+        <is>
+          <t>MetaGPT</t>
+        </is>
+      </c>
+      <c r="I81" s="5" t="inlineStr">
+        <is>
+          <t>@MetaGPT_ / GitHub</t>
+        </is>
+      </c>
+      <c r="J81" s="5" t="inlineStr">
+        <is>
+          <t>GitHub / company</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="4" t="inlineStr">
+        <is>
+          <t>Med</t>
+        </is>
+      </c>
+      <c r="B82" s="5" t="inlineStr">
+        <is>
+          <t>A. Framework &amp; Infra Builders</t>
+        </is>
+      </c>
+      <c r="C82" s="6" t="inlineStr">
+        <is>
+          <t>Dify team (张路宇 / LangGenius)</t>
+        </is>
+      </c>
+      <c r="D82" s="5" t="inlineStr">
+        <is>
+          <t>Dify — open-source LLM app &amp; agent platform</t>
+        </is>
+      </c>
+      <c r="E82" s="5" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="F82" s="5" t="inlineStr">
+        <is>
+          <t>Dify is one of the most-used OSS agent/LLM-app dev platforms worldwide</t>
+        </is>
+      </c>
+      <c r="G82" s="5" t="inlineStr">
+        <is>
+          <t>Agent-building infra widely adopted in CN + globally</t>
+        </is>
+      </c>
+      <c r="H82" s="5" t="inlineStr">
+        <is>
+          <t>Dify</t>
+        </is>
+      </c>
+      <c r="I82" s="5" t="inlineStr">
+        <is>
+          <t>@dify_ai (verify) / GitHub</t>
+        </is>
+      </c>
+      <c r="J82" s="5" t="inlineStr">
+        <is>
+          <t>GitHub / company</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="inlineStr">
+        <is>
+          <t>Med</t>
+        </is>
+      </c>
+      <c r="B83" s="5" t="inlineStr">
+        <is>
+          <t>A. Framework &amp; Infra Builders</t>
+        </is>
+      </c>
+      <c r="C83" s="6" t="inlineStr">
+        <is>
+          <t>Guohao Li (李国豪)</t>
+        </is>
+      </c>
+      <c r="D83" s="5" t="inlineStr">
+        <is>
+          <t>CAMEL-AI / Eigent — Founder</t>
+        </is>
+      </c>
+      <c r="E83" s="5" t="inlineStr">
+        <is>
+          <t>CN/UK</t>
+        </is>
+      </c>
+      <c r="F83" s="5" t="inlineStr">
+        <is>
+          <t>CAMEL = pioneering 'communicative agents' multi-agent OSS framework</t>
+        </is>
+      </c>
+      <c r="G83" s="5" t="inlineStr">
+        <is>
+          <t>Agent-to-agent communication research; diaspora bridge</t>
+        </is>
+      </c>
+      <c r="H83" s="5" t="inlineStr">
+        <is>
+          <t>CAMEL-AI</t>
+        </is>
+      </c>
+      <c r="I83" s="5" t="inlineStr">
+        <is>
+          <t>@lgh_xxh (verify) / camel-ai.org</t>
+        </is>
+      </c>
+      <c r="J83" s="5" t="inlineStr">
+        <is>
+          <t>X / GitHub</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="4" t="inlineStr">
+        <is>
+          <t>Med</t>
+        </is>
+      </c>
+      <c r="B84" s="5" t="inlineStr">
+        <is>
+          <t>A. Framework &amp; Infra Builders</t>
+        </is>
+      </c>
+      <c r="C84" s="6" t="inlineStr">
+        <is>
+          <t>ByteDance Coze (扣子) team</t>
+        </is>
+      </c>
+      <c r="D84" s="5" t="inlineStr">
+        <is>
+          <t>ByteDance — Coze agent-building platform</t>
+        </is>
+      </c>
+      <c r="E84" s="5" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="F84" s="5" t="inlineStr">
+        <is>
+          <t>Coze = mass-market no-code agent/bot builder (CN 扣子 + intl)</t>
+        </is>
+      </c>
+      <c r="G84" s="5" t="inlineStr">
+        <is>
+          <t>Consumer 'build your own agent' platform; distribution comp</t>
+        </is>
+      </c>
+      <c r="H84" s="5" t="inlineStr">
+        <is>
+          <t>Coze / 扣子</t>
+        </is>
+      </c>
+      <c r="I84" s="5" t="inlineStr">
+        <is>
+          <t>coze.com</t>
+        </is>
+      </c>
+      <c r="J84" s="5" t="inlineStr">
+        <is>
+          <t>Company / BD</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="4" t="inlineStr">
+        <is>
+          <t>Med</t>
+        </is>
+      </c>
+      <c r="B85" s="5" t="inlineStr">
+        <is>
+          <t>A. Framework &amp; Infra Builders</t>
+        </is>
+      </c>
+      <c r="C85" s="6" t="inlineStr">
+        <is>
+          <t>Zhou Jingren (周靖人)</t>
+        </is>
+      </c>
+      <c r="D85" s="5" t="inlineStr">
+        <is>
+          <t>Alibaba — CTO, Alibaba Cloud (Qwen / AgentScope)</t>
+        </is>
+      </c>
+      <c r="E85" s="5" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="F85" s="5" t="inlineStr">
+        <is>
+          <t>Leads Qwen + Qwen-Agent + AgentScope multi-agent platform</t>
+        </is>
+      </c>
+      <c r="G85" s="5" t="inlineStr">
+        <is>
+          <t>Open model + agent framework backbone in CN</t>
+        </is>
+      </c>
+      <c r="H85" s="5" t="inlineStr">
+        <is>
+          <t>Qwen-Agent, AgentScope</t>
+        </is>
+      </c>
+      <c r="I85" s="5" t="inlineStr">
+        <is>
+          <t>Alibaba Cloud</t>
+        </is>
+      </c>
+      <c r="J85" s="5" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B86" s="8" t="inlineStr">
+        <is>
+          <t>B. Agent Startup Founders</t>
+        </is>
+      </c>
+      <c r="C86" s="9" t="inlineStr">
+        <is>
+          <t>Jing Kun (景鲲)</t>
+        </is>
+      </c>
+      <c r="D86" s="8" t="inlineStr">
+        <is>
+          <t>Genspark (MainFunc) — Co-founder &amp; CEO (ex-Baidu)</t>
+        </is>
+      </c>
+      <c r="E86" s="8" t="inlineStr">
+        <is>
+          <t>CN/US</t>
+        </is>
+      </c>
+      <c r="F86" s="8" t="inlineStr">
+        <is>
+          <t>Genspark = fast-rising agentic search / all-in-one 'AI agent' product</t>
+        </is>
+      </c>
+      <c r="G86" s="8" t="inlineStr">
+        <is>
+          <t>General consumer agent; closest CN-founded product comp to iLands assistant layer</t>
+        </is>
+      </c>
+      <c r="H86" s="8" t="inlineStr">
+        <is>
+          <t>Genspark</t>
+        </is>
+      </c>
+      <c r="I86" s="8" t="inlineStr">
+        <is>
+          <t>@JingKun (verify)</t>
+        </is>
+      </c>
+      <c r="J86" s="8" t="inlineStr">
+        <is>
+          <t>X / company</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="7" t="inlineStr">
+        <is>
+          <t>Med</t>
+        </is>
+      </c>
+      <c r="B87" s="8" t="inlineStr">
+        <is>
+          <t>B. Agent Startup Founders</t>
+        </is>
+      </c>
+      <c r="C87" s="9" t="inlineStr">
+        <is>
+          <t>Xie Yang (谢扬)</t>
+        </is>
+      </c>
+      <c r="D87" s="8" t="inlineStr">
+        <is>
+          <t>Fellou — Founder</t>
+        </is>
+      </c>
+      <c r="E87" s="8" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="F87" s="8" t="inlineStr">
+        <is>
+          <t>Fellou = 'agentic browser' that takes actions for users</t>
+        </is>
+      </c>
+      <c r="G87" s="8" t="inlineStr">
+        <is>
+          <t>Web-action personal agent; CN consumer angle</t>
+        </is>
+      </c>
+      <c r="H87" s="8" t="inlineStr">
+        <is>
+          <t>Fellou</t>
+        </is>
+      </c>
+      <c r="I87" s="8" t="inlineStr">
+        <is>
+          <t>fellou.ai</t>
+        </is>
+      </c>
+      <c r="J87" s="8" t="inlineStr">
+        <is>
+          <t>Company / X</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="7" t="inlineStr">
+        <is>
+          <t>Med</t>
+        </is>
+      </c>
+      <c r="B88" s="8" t="inlineStr">
+        <is>
+          <t>B. Agent Startup Founders</t>
+        </is>
+      </c>
+      <c r="C88" s="9" t="inlineStr">
+        <is>
+          <t>Zhou Jian (周健)</t>
+        </is>
+      </c>
+      <c r="D88" s="8" t="inlineStr">
+        <is>
+          <t>Lanma Tech (澜码科技) — Founder &amp; CEO</t>
+        </is>
+      </c>
+      <c r="E88" s="8" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="F88" s="8" t="inlineStr">
+        <is>
+          <t>Enterprise agent platform (AskXBOT) for Chinese businesses</t>
+        </is>
+      </c>
+      <c r="G88" s="8" t="inlineStr">
+        <is>
+          <t>Enterprise agent GTM in CN market</t>
+        </is>
+      </c>
+      <c r="H88" s="8" t="inlineStr">
+        <is>
+          <t>澜码 AskXBOT</t>
+        </is>
+      </c>
+      <c r="I88" s="8" t="inlineStr">
+        <is>
+          <t>company site</t>
+        </is>
+      </c>
+      <c r="J88" s="8" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="10" t="inlineStr">
+        <is>
+          <t>★High</t>
+        </is>
+      </c>
+      <c r="B89" s="11" t="inlineStr">
+        <is>
+          <t>C. Researchers &amp; Academics</t>
+        </is>
+      </c>
+      <c r="C89" s="12" t="inlineStr">
+        <is>
+          <t>Qiu Xipeng (邱锡鹏)</t>
+        </is>
+      </c>
+      <c r="D89" s="11" t="inlineStr">
+        <is>
+          <t>Fudan University — NLP prof (MOSS)</t>
+        </is>
+      </c>
+      <c r="E89" s="11" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="F89" s="11" t="inlineStr">
+        <is>
+          <t>Led MOSS; senior author of 'The Rise and Potential of LLM-based Agents: A Survey'</t>
+        </is>
+      </c>
+      <c r="G89" s="11" t="inlineStr">
+        <is>
+          <t>The canonical CN academic map of LLM agents — research credibility &amp; advisory</t>
+        </is>
+      </c>
+      <c r="H89" s="11" t="inlineStr">
+        <is>
+          <t>LLM-Agents Survey, MOSS</t>
+        </is>
+      </c>
+      <c r="I89" s="11" t="inlineStr">
+        <is>
+          <t>Fudan / GitHub</t>
+        </is>
+      </c>
+      <c r="J89" s="11" t="inlineStr">
+        <is>
+          <t>Academic email</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="13" t="inlineStr">
+        <is>
+          <t>Med</t>
+        </is>
+      </c>
+      <c r="B90" s="11" t="inlineStr">
+        <is>
+          <t>C. Researchers &amp; Academics</t>
+        </is>
+      </c>
+      <c r="C90" s="12" t="inlineStr">
+        <is>
+          <t>Huang Minlie (黄民烈)</t>
+        </is>
+      </c>
+      <c r="D90" s="11" t="inlineStr">
+        <is>
+          <t>Tsinghua University — CoAI; Lingxin (聆心智能)</t>
+        </is>
+      </c>
+      <c r="E90" s="11" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="F90" s="11" t="inlineStr">
+        <is>
+          <t>Dialogue systems &amp; emotional/companion agents; founded a persona-AI company</t>
+        </is>
+      </c>
+      <c r="G90" s="11" t="inlineStr">
+        <is>
+          <t>Companion/persona agents = adjacent to 'live with your AI'</t>
+        </is>
+      </c>
+      <c r="H90" s="11" t="inlineStr">
+        <is>
+          <t>CoAI, ChatGLM dialog</t>
+        </is>
+      </c>
+      <c r="I90" s="11" t="inlineStr">
+        <is>
+          <t>Tsinghua</t>
+        </is>
+      </c>
+      <c r="J90" s="11" t="inlineStr">
+        <is>
+          <t>Academic / company</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="13" t="inlineStr">
+        <is>
+          <t>Med</t>
+        </is>
+      </c>
+      <c r="B91" s="11" t="inlineStr">
+        <is>
+          <t>C. Researchers &amp; Academics</t>
+        </is>
+      </c>
+      <c r="C91" s="12" t="inlineStr">
+        <is>
+          <t>Sun Maosong (孙茂松)</t>
+        </is>
+      </c>
+      <c r="D91" s="11" t="inlineStr">
+        <is>
+          <t>Tsinghua University — NLP; OpenBMB advisor</t>
+        </is>
+      </c>
+      <c r="E91" s="11" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="F91" s="11" t="inlineStr">
+        <is>
+          <t>Senior figure behind Tsinghua NLP + OpenBMB (AgentVerse/ChatDev lineage)</t>
+        </is>
+      </c>
+      <c r="G91" s="11" t="inlineStr">
+        <is>
+          <t>Multi-agent OSS ecosystem gravity in CN academia</t>
+        </is>
+      </c>
+      <c r="H91" s="11" t="inlineStr">
+        <is>
+          <t>OpenBMB, THUNLP</t>
+        </is>
+      </c>
+      <c r="I91" s="11" t="inlineStr">
+        <is>
+          <t>Tsinghua</t>
+        </is>
+      </c>
+      <c r="J91" s="11" t="inlineStr">
+        <is>
+          <t>Academic</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="13" t="inlineStr">
+        <is>
+          <t>Med</t>
+        </is>
+      </c>
+      <c r="B92" s="11" t="inlineStr">
+        <is>
+          <t>C. Researchers &amp; Academics</t>
+        </is>
+      </c>
+      <c r="C92" s="12" t="inlineStr">
+        <is>
+          <t>Junyang Lin (林俊旸)</t>
+        </is>
+      </c>
+      <c r="D92" s="11" t="inlineStr">
+        <is>
+          <t>Alibaba — Qwen tech lead</t>
+        </is>
+      </c>
+      <c r="E92" s="11" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="F92" s="11" t="inlineStr">
+        <is>
+          <t>Drives Qwen models + Qwen-Agent; very active bilingual voice</t>
+        </is>
+      </c>
+      <c r="G92" s="11" t="inlineStr">
+        <is>
+          <t>Open model + agent tooling; reachable on X</t>
+        </is>
+      </c>
+      <c r="H92" s="11" t="inlineStr">
+        <is>
+          <t>Qwen, Qwen-Agent</t>
+        </is>
+      </c>
+      <c r="I92" s="11" t="inlineStr">
+        <is>
+          <t>@JustinLin610 (X)</t>
+        </is>
+      </c>
+      <c r="J92" s="11" t="inlineStr">
+        <is>
+          <t>X DM</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="14" t="inlineStr">
+        <is>
+          <t>★High</t>
+        </is>
+      </c>
+      <c r="B93" s="15" t="inlineStr">
+        <is>
+          <t>D. Investors &amp; VCs</t>
+        </is>
+      </c>
+      <c r="C93" s="16" t="inlineStr">
+        <is>
+          <t>Qi Lu (陆奇)</t>
+        </is>
+      </c>
+      <c r="D93" s="15" t="inlineStr">
+        <is>
+          <t>MiraclePlus (奇绩创坛) — Founder &amp; CEO (ex-Baidu COO, ex-MSFT EVP)</t>
+        </is>
+      </c>
+      <c r="E93" s="15" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="F93" s="15" t="inlineStr">
+        <is>
+          <t>Most respected AI operator-investor in CN; his 'large-model worldview' talks set the agenda</t>
+        </is>
+      </c>
+      <c r="G93" s="15" t="inlineStr">
+        <is>
+          <t>Top thesis ally + door-opener across CN AI; also a thought leader</t>
+        </is>
+      </c>
+      <c r="H93" s="15" t="inlineStr">
+        <is>
+          <t>奇绩 '大模型世界观' 演讲</t>
+        </is>
+      </c>
+      <c r="I93" s="15" t="inlineStr">
+        <is>
+          <t>MiraclePlus</t>
+        </is>
+      </c>
+      <c r="J93" s="15" t="inlineStr">
+        <is>
+          <t>Warm intro</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="17" t="inlineStr">
+        <is>
+          <t>Med</t>
+        </is>
+      </c>
+      <c r="B94" s="15" t="inlineStr">
+        <is>
+          <t>D. Investors &amp; VCs</t>
+        </is>
+      </c>
+      <c r="C94" s="16" t="inlineStr">
+        <is>
+          <t>Zhu Xiaohu (朱啸虎)</t>
+        </is>
+      </c>
+      <c r="D94" s="15" t="inlineStr">
+        <is>
+          <t>GSR Ventures (金沙江创投) — Managing Partner</t>
+        </is>
+      </c>
+      <c r="E94" s="15" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="F94" s="15" t="inlineStr">
+        <is>
+          <t>Loudest CN VC voice on AI-application &amp; agent商业化 (and its skeptics)</t>
+        </is>
+      </c>
+      <c r="G94" s="15" t="inlineStr">
+        <is>
+          <t>High-signal (and provocative) CN application-layer investor</t>
+        </is>
+      </c>
+      <c r="H94" s="15" t="inlineStr">
+        <is>
+          <t>GSR / public debates</t>
+        </is>
+      </c>
+      <c r="I94" s="15" t="inlineStr">
+        <is>
+          <t>公开采访 / 36氪</t>
+        </is>
+      </c>
+      <c r="J94" s="15" t="inlineStr">
+        <is>
+          <t>Warm intro</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="17" t="inlineStr">
+        <is>
+          <t>Med</t>
+        </is>
+      </c>
+      <c r="B95" s="15" t="inlineStr">
+        <is>
+          <t>D. Investors &amp; VCs</t>
+        </is>
+      </c>
+      <c r="C95" s="16" t="inlineStr">
+        <is>
+          <t>Qu Kai (曲凯)</t>
+        </is>
+      </c>
+      <c r="D95" s="15" t="inlineStr">
+        <is>
+          <t>42Zhang Jing (42章经) — Founder; VC &amp; top AI podcast</t>
+        </is>
+      </c>
+      <c r="E95" s="15" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="F95" s="15" t="inlineStr">
+        <is>
+          <t>Runs 42章经 — a leading CN VC newsletter + AI podcast; investor-media hybrid</t>
+        </is>
+      </c>
+      <c r="G95" s="15" t="inlineStr">
+        <is>
+          <t>Investor + best CN AI-founder podcast — dual value</t>
+        </is>
+      </c>
+      <c r="H95" s="15" t="inlineStr">
+        <is>
+          <t>42章经 podcast</t>
+        </is>
+      </c>
+      <c r="I95" s="15" t="inlineStr">
+        <is>
+          <t>公众号 42章经</t>
+        </is>
+      </c>
+      <c r="J95" s="15" t="inlineStr">
+        <is>
+          <t>WeChat / podcast pitch</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="18" t="inlineStr">
+        <is>
+          <t>★High</t>
+        </is>
+      </c>
+      <c r="B96" s="19" t="inlineStr">
+        <is>
+          <t>E. Thought Leaders &amp; Media</t>
+        </is>
+      </c>
+      <c r="C96" s="20" t="inlineStr">
+        <is>
+          <t>Zhang Xiaojun (张小珺)</t>
+        </is>
+      </c>
+      <c r="D96" s="19" t="inlineStr">
+        <is>
+          <t>Tencent News — '商业访谈录' host</t>
+        </is>
+      </c>
+      <c r="E96" s="19" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="F96" s="19" t="inlineStr">
+        <is>
+          <t>Deepest long-form CN interviews with AI founders &amp; researchers</t>
+        </is>
+      </c>
+      <c r="G96" s="19" t="inlineStr">
+        <is>
+          <t>The premier CN platform to tell the iLands story to insiders</t>
+        </is>
+      </c>
+      <c r="H96" s="19" t="inlineStr">
+        <is>
+          <t>《商业访谈录》podcast</t>
+        </is>
+      </c>
+      <c r="I96" s="19" t="inlineStr">
+        <is>
+          <t>腾讯新闻 / 小宇宙</t>
+        </is>
+      </c>
+      <c r="J96" s="19" t="inlineStr">
+        <is>
+          <t>Pitch producer</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="21" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B97" s="19" t="inlineStr">
+        <is>
+          <t>E. Thought Leaders &amp; Media</t>
+        </is>
+      </c>
+      <c r="C97" s="20" t="inlineStr">
+        <is>
+          <t>Zhang Peng (张鹏)</t>
+        </is>
+      </c>
+      <c r="D97" s="19" t="inlineStr">
+        <is>
+          <t>GeekPark (极客公园) — Founder</t>
+        </is>
+      </c>
+      <c r="E97" s="19" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="F97" s="19" t="inlineStr">
+        <is>
+          <t>GeekPark = top CN tech-founder media &amp; events (AGI Playground)</t>
+        </is>
+      </c>
+      <c r="G97" s="19" t="inlineStr">
+        <is>
+          <t>Media + stage to reach CN AI ecosystem</t>
+        </is>
+      </c>
+      <c r="H97" s="19" t="inlineStr">
+        <is>
+          <t>极客公园 / Founder Park</t>
+        </is>
+      </c>
+      <c r="I97" s="19" t="inlineStr">
+        <is>
+          <t>公众号 极客公园</t>
+        </is>
+      </c>
+      <c r="J97" s="19" t="inlineStr">
+        <is>
+          <t>Media pitch</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="21" t="inlineStr">
+        <is>
+          <t>Med</t>
+        </is>
+      </c>
+      <c r="B98" s="19" t="inlineStr">
+        <is>
+          <t>E. Thought Leaders &amp; Media</t>
+        </is>
+      </c>
+      <c r="C98" s="20" t="inlineStr">
+        <is>
+          <t>LatePost (晚点) team</t>
+        </is>
+      </c>
+      <c r="D98" s="19" t="inlineStr">
+        <is>
+          <t>LatePost (晚点LatePost) — tech business media</t>
+        </is>
+      </c>
+      <c r="E98" s="19" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="F98" s="19" t="inlineStr">
+        <is>
+          <t>Breaks the biggest CN AI company/funding stories</t>
+        </is>
+      </c>
+      <c r="G98" s="19" t="inlineStr">
+        <is>
+          <t>Press for CN milestones &amp; positioning</t>
+        </is>
+      </c>
+      <c r="H98" s="19" t="inlineStr">
+        <is>
+          <t>晚点LatePost</t>
+        </is>
+      </c>
+      <c r="I98" s="19" t="inlineStr">
+        <is>
+          <t>公众号 晚点</t>
+        </is>
+      </c>
+      <c r="J98" s="19" t="inlineStr">
+        <is>
+          <t>Email pitch</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:J80"/>
+  <autoFilter ref="A4:J98"/>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>

</xml_diff>

<commit_message>
Add Coverage & Reading List sheet: 108 verified links across 75 people
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012LRydPx3p71npFqtrfS6Ef
</commit_message>
<xml_diff>
--- a/iLands_Agent_Economy_Network_2026-07-01.xlsx
+++ b/iLands_Agent_Economy_Network_2026-07-01.xlsx
@@ -8,10 +8,12 @@
   </bookViews>
   <sheets>
     <sheet name="Agent Economy Network" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="How to use" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Coverage &amp; Reading List" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="How to use" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Agent Economy Network'!$A$4:$J$98</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Coverage &amp; Reading List'!$A$4:$F$112</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -59,8 +61,23 @@
       <b val="1"/>
       <sz val="12"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00555555"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <color rgb="001155CC"/>
+      <sz val="9"/>
+      <u val="single"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -117,6 +134,16 @@
         <fgColor rgb="00FFF0E6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F7F9FC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -144,7 +171,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -248,6 +275,52 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -5598,6 +5671,3645 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F112"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="37" t="inlineStr">
+        <is>
+          <t>iLands · Agent-Economy Network — Coverage &amp; Reading List</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="38" t="inlineStr">
+        <is>
+          <t>Signature works, key interviews, papers &amp; podcasts per person. All links agent-verified as live (2026-07-01); a few paywalled/bot-blocked outlets (Forbes/Bloomberg/VentureBeat) are real but were not machine-fetched. Own-work/landmark items listed first per person.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="39" t="inlineStr">
+        <is>
+          <t>Person</t>
+        </is>
+      </c>
+      <c r="B4" s="39" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C4" s="39" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="D4" s="39" t="inlineStr">
+        <is>
+          <t>Outlet / Venue</t>
+        </is>
+      </c>
+      <c r="E4" s="39" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="F4" s="39" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="40" t="inlineStr">
+        <is>
+          <t>Joon Sung Park</t>
+        </is>
+      </c>
+      <c r="B5" s="41" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C5" s="42" t="inlineStr">
+        <is>
+          <t>Generative Agents: Interactive Simulacra of Human Behavior</t>
+        </is>
+      </c>
+      <c r="D5" s="42" t="inlineStr">
+        <is>
+          <t>arXiv (UIST 2023)</t>
+        </is>
+      </c>
+      <c r="E5" s="42" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="F5" s="43" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2304.03442</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="40" t="inlineStr">
+        <is>
+          <t>Joon Sung Park</t>
+        </is>
+      </c>
+      <c r="B6" s="44" t="inlineStr">
+        <is>
+          <t>Podcast</t>
+        </is>
+      </c>
+      <c r="C6" s="42" t="inlineStr">
+        <is>
+          <t>Simulating Humans at Scale: Simile's Joon Sung Park</t>
+        </is>
+      </c>
+      <c r="D6" s="42" t="inlineStr">
+        <is>
+          <t>Sequoia Training Data</t>
+        </is>
+      </c>
+      <c r="E6" s="42" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F6" s="43" t="inlineStr">
+        <is>
+          <t>https://sequoiacap.com/podcast/simulating-humans-at-scale-similes-joon-sung-park/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="40" t="inlineStr">
+        <is>
+          <t>Joon Sung Park</t>
+        </is>
+      </c>
+      <c r="B7" s="44" t="inlineStr">
+        <is>
+          <t>Podcast</t>
+        </is>
+      </c>
+      <c r="C7" s="42" t="inlineStr">
+        <is>
+          <t>Modeling Human Behavior with Generative Agents</t>
+        </is>
+      </c>
+      <c r="D7" s="42" t="inlineStr">
+        <is>
+          <t>TWIML AI Podcast</t>
+        </is>
+      </c>
+      <c r="E7" s="42" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="F7" s="43" t="inlineStr">
+        <is>
+          <t>https://twimlai.com/podcast/twimlai/modeling-human-behavior-with-generative-agents</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="45" t="inlineStr">
+        <is>
+          <t>Michael S. Bernstein</t>
+        </is>
+      </c>
+      <c r="B8" s="41" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C8" s="46" t="inlineStr">
+        <is>
+          <t>Generative Agents: Interactive Simulacra of Human Behavior</t>
+        </is>
+      </c>
+      <c r="D8" s="46" t="inlineStr">
+        <is>
+          <t>arXiv (UIST 2023)</t>
+        </is>
+      </c>
+      <c r="E8" s="46" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="F8" s="47" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2304.03442</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="45" t="inlineStr">
+        <is>
+          <t>Michael S. Bernstein</t>
+        </is>
+      </c>
+      <c r="B9" s="48" t="inlineStr">
+        <is>
+          <t>Press</t>
+        </is>
+      </c>
+      <c r="C9" s="46" t="inlineStr">
+        <is>
+          <t>AI agents simulate 1,052 individuals' personalities with impressive accuracy</t>
+        </is>
+      </c>
+      <c r="D9" s="46" t="inlineStr">
+        <is>
+          <t>Stanford HAI</t>
+        </is>
+      </c>
+      <c r="E9" s="46" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F9" s="47" t="inlineStr">
+        <is>
+          <t>https://hai.stanford.edu/news/ai-agents-simulate-1052-individuals-personalities-impressive-accuracy</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="40" t="inlineStr">
+        <is>
+          <t>Jim Fan</t>
+        </is>
+      </c>
+      <c r="B10" s="41" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C10" s="42" t="inlineStr">
+        <is>
+          <t>Eureka: Human-Level Reward Design via Coding Large Language Models</t>
+        </is>
+      </c>
+      <c r="D10" s="42" t="inlineStr">
+        <is>
+          <t>arXiv</t>
+        </is>
+      </c>
+      <c r="E10" s="42" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="F10" s="43" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2310.12931</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="40" t="inlineStr">
+        <is>
+          <t>Jim Fan</t>
+        </is>
+      </c>
+      <c r="B11" s="49" t="inlineStr">
+        <is>
+          <t>Talk</t>
+        </is>
+      </c>
+      <c r="C11" s="42" t="inlineStr">
+        <is>
+          <t>The next grand challenge for AI</t>
+        </is>
+      </c>
+      <c r="D11" s="42" t="inlineStr">
+        <is>
+          <t>TED</t>
+        </is>
+      </c>
+      <c r="E11" s="42" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F11" s="43" t="inlineStr">
+        <is>
+          <t>https://www.ted.com/talks/jim_fan_the_next_grand_challenge_for_ai</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="40" t="inlineStr">
+        <is>
+          <t>Jim Fan</t>
+        </is>
+      </c>
+      <c r="B12" s="44" t="inlineStr">
+        <is>
+          <t>Podcast</t>
+        </is>
+      </c>
+      <c r="C12" s="42" t="inlineStr">
+        <is>
+          <t>Nvidia's Jim Fan on Robots Thinking Fast and Slow</t>
+        </is>
+      </c>
+      <c r="D12" s="42" t="inlineStr">
+        <is>
+          <t>Sequoia Training Data</t>
+        </is>
+      </c>
+      <c r="E12" s="42" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F12" s="43" t="inlineStr">
+        <is>
+          <t>https://sequoiacap.com/podcast/training-data-jim-fan/</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="45" t="inlineStr">
+        <is>
+          <t>Guanzhi Wang</t>
+        </is>
+      </c>
+      <c r="B13" s="41" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C13" s="46" t="inlineStr">
+        <is>
+          <t>Voyager: An Open-Ended Embodied Agent with Large Language Models</t>
+        </is>
+      </c>
+      <c r="D13" s="46" t="inlineStr">
+        <is>
+          <t>arXiv</t>
+        </is>
+      </c>
+      <c r="E13" s="46" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="F13" s="47" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2305.16291</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="45" t="inlineStr">
+        <is>
+          <t>Guanzhi Wang</t>
+        </is>
+      </c>
+      <c r="B14" s="48" t="inlineStr">
+        <is>
+          <t>Press</t>
+        </is>
+      </c>
+      <c r="C14" s="46" t="inlineStr">
+        <is>
+          <t>Open-Ended AI Agent Voyager Autonomously Plays Minecraft</t>
+        </is>
+      </c>
+      <c r="D14" s="46" t="inlineStr">
+        <is>
+          <t>NVIDIA Blog</t>
+        </is>
+      </c>
+      <c r="E14" s="46" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="F14" s="47" t="inlineStr">
+        <is>
+          <t>https://blogs.nvidia.com/blog/ai-jim-fan/</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="40" t="inlineStr">
+        <is>
+          <t>Jeff Clune</t>
+        </is>
+      </c>
+      <c r="B15" s="41" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C15" s="42" t="inlineStr">
+        <is>
+          <t>Paired Open-Ended Trailblazer (POET)</t>
+        </is>
+      </c>
+      <c r="D15" s="42" t="inlineStr">
+        <is>
+          <t>arXiv</t>
+        </is>
+      </c>
+      <c r="E15" s="42" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="F15" s="43" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/1901.01753</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="40" t="inlineStr">
+        <is>
+          <t>Jeff Clune</t>
+        </is>
+      </c>
+      <c r="B16" s="44" t="inlineStr">
+        <is>
+          <t>Podcast</t>
+        </is>
+      </c>
+      <c r="C16" s="42" t="inlineStr">
+        <is>
+          <t>Jeff Clune (AI-GAs, POET, Open-Endedness)</t>
+        </is>
+      </c>
+      <c r="D16" s="42" t="inlineStr">
+        <is>
+          <t>TalkRL</t>
+        </is>
+      </c>
+      <c r="E16" s="42" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="F16" s="43" t="inlineStr">
+        <is>
+          <t>https://www.talkrl.com/episodes/jeff-clune</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="40" t="inlineStr">
+        <is>
+          <t>Jeff Clune</t>
+        </is>
+      </c>
+      <c r="B17" s="49" t="inlineStr">
+        <is>
+          <t>Talk</t>
+        </is>
+      </c>
+      <c r="C17" s="42" t="inlineStr">
+        <is>
+          <t>Open-Ended and AI-Generating Algorithms in the Era of Foundation Models</t>
+        </is>
+      </c>
+      <c r="D17" s="42" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="E17" s="42" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F17" s="43" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=tP5AB5GgZAE</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="45" t="inlineStr">
+        <is>
+          <t>Tim Rocktäschel</t>
+        </is>
+      </c>
+      <c r="B18" s="41" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C18" s="46" t="inlineStr">
+        <is>
+          <t>Open-Endedness is Essential for Artificial Superhuman Intelligence</t>
+        </is>
+      </c>
+      <c r="D18" s="46" t="inlineStr">
+        <is>
+          <t>arXiv (ICML 2024)</t>
+        </is>
+      </c>
+      <c r="E18" s="46" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F18" s="47" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2406.04268</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="40" t="inlineStr">
+        <is>
+          <t>Shunyu Yao</t>
+        </is>
+      </c>
+      <c r="B19" s="41" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C19" s="42" t="inlineStr">
+        <is>
+          <t>ReAct: Synergizing Reasoning and Acting in Language Models</t>
+        </is>
+      </c>
+      <c r="D19" s="42" t="inlineStr">
+        <is>
+          <t>arXiv</t>
+        </is>
+      </c>
+      <c r="E19" s="42" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="F19" s="43" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2210.03629</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="40" t="inlineStr">
+        <is>
+          <t>Shunyu Yao</t>
+        </is>
+      </c>
+      <c r="B20" s="41" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C20" s="42" t="inlineStr">
+        <is>
+          <t>Tree of Thoughts: Deliberate Problem Solving with Large Language Models</t>
+        </is>
+      </c>
+      <c r="D20" s="42" t="inlineStr">
+        <is>
+          <t>arXiv</t>
+        </is>
+      </c>
+      <c r="E20" s="42" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="F20" s="43" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2305.10601</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="40" t="inlineStr">
+        <is>
+          <t>Shunyu Yao</t>
+        </is>
+      </c>
+      <c r="B21" s="44" t="inlineStr">
+        <is>
+          <t>Podcast</t>
+        </is>
+      </c>
+      <c r="C21" s="42" t="inlineStr">
+        <is>
+          <t>Language Agents: From Reasoning to Acting</t>
+        </is>
+      </c>
+      <c r="D21" s="42" t="inlineStr">
+        <is>
+          <t>Latent Space</t>
+        </is>
+      </c>
+      <c r="E21" s="42" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F21" s="43" t="inlineStr">
+        <is>
+          <t>https://www.latent.space/p/shunyu</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="45" t="inlineStr">
+        <is>
+          <t>Noah Shinn</t>
+        </is>
+      </c>
+      <c r="B22" s="41" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C22" s="46" t="inlineStr">
+        <is>
+          <t>Reflexion: Language Agents with Verbal Reinforcement Learning</t>
+        </is>
+      </c>
+      <c r="D22" s="46" t="inlineStr">
+        <is>
+          <t>arXiv (NeurIPS 2023)</t>
+        </is>
+      </c>
+      <c r="E22" s="46" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="F22" s="47" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2303.11366</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="40" t="inlineStr">
+        <is>
+          <t>Ofir Press</t>
+        </is>
+      </c>
+      <c r="B23" s="41" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C23" s="42" t="inlineStr">
+        <is>
+          <t>SWE-bench: Can Language Models Resolve Real-World GitHub Issues?</t>
+        </is>
+      </c>
+      <c r="D23" s="42" t="inlineStr">
+        <is>
+          <t>arXiv</t>
+        </is>
+      </c>
+      <c r="E23" s="42" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="F23" s="43" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2310.06770</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="40" t="inlineStr">
+        <is>
+          <t>Ofir Press</t>
+        </is>
+      </c>
+      <c r="B24" s="41" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C24" s="42" t="inlineStr">
+        <is>
+          <t>SWE-agent: Agent-Computer Interfaces Enable Automated Software Engineering</t>
+        </is>
+      </c>
+      <c r="D24" s="42" t="inlineStr">
+        <is>
+          <t>arXiv</t>
+        </is>
+      </c>
+      <c r="E24" s="42" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F24" s="43" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2405.15793</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="45" t="inlineStr">
+        <is>
+          <t>Yu Su</t>
+        </is>
+      </c>
+      <c r="B25" s="41" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C25" s="46" t="inlineStr">
+        <is>
+          <t>Mind2Web: Towards a Generalist Agent for the Web</t>
+        </is>
+      </c>
+      <c r="D25" s="46" t="inlineStr">
+        <is>
+          <t>arXiv (NeurIPS 2023)</t>
+        </is>
+      </c>
+      <c r="E25" s="46" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="F25" s="47" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2306.06070</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="40" t="inlineStr">
+        <is>
+          <t>Xingyao Wang</t>
+        </is>
+      </c>
+      <c r="B26" s="41" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C26" s="42" t="inlineStr">
+        <is>
+          <t>OpenHands: An Open Platform for AI Software Developers as Generalist Agents</t>
+        </is>
+      </c>
+      <c r="D26" s="42" t="inlineStr">
+        <is>
+          <t>arXiv (ICLR 2025)</t>
+        </is>
+      </c>
+      <c r="E26" s="42" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F26" s="43" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2407.16741</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="45" t="inlineStr">
+        <is>
+          <t>Denny Zhou</t>
+        </is>
+      </c>
+      <c r="B27" s="41" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C27" s="46" t="inlineStr">
+        <is>
+          <t>Chain-of-Thought Prompting Elicits Reasoning in Large Language Models</t>
+        </is>
+      </c>
+      <c r="D27" s="46" t="inlineStr">
+        <is>
+          <t>arXiv</t>
+        </is>
+      </c>
+      <c r="E27" s="46" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="F27" s="47" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2201.11903</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="45" t="inlineStr">
+        <is>
+          <t>Denny Zhou</t>
+        </is>
+      </c>
+      <c r="B28" s="41" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C28" s="46" t="inlineStr">
+        <is>
+          <t>Self-Consistency Improves Chain of Thought Reasoning</t>
+        </is>
+      </c>
+      <c r="D28" s="46" t="inlineStr">
+        <is>
+          <t>arXiv</t>
+        </is>
+      </c>
+      <c r="E28" s="46" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="F28" s="47" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2203.11171</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="40" t="inlineStr">
+        <is>
+          <t>Percy Liang</t>
+        </is>
+      </c>
+      <c r="B29" s="41" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C29" s="42" t="inlineStr">
+        <is>
+          <t>Holistic Evaluation of Language Models (HELM)</t>
+        </is>
+      </c>
+      <c r="D29" s="42" t="inlineStr">
+        <is>
+          <t>arXiv</t>
+        </is>
+      </c>
+      <c r="E29" s="42" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="F29" s="43" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2211.09110</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="40" t="inlineStr">
+        <is>
+          <t>Percy Liang</t>
+        </is>
+      </c>
+      <c r="B30" s="44" t="inlineStr">
+        <is>
+          <t>Podcast</t>
+        </is>
+      </c>
+      <c r="C30" s="42" t="inlineStr">
+        <is>
+          <t>Percy Liang on the paradigm shift and societal effects of foundation models</t>
+        </is>
+      </c>
+      <c r="D30" s="42" t="inlineStr">
+        <is>
+          <t>Imbue Podcast</t>
+        </is>
+      </c>
+      <c r="E30" s="42" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F30" s="43" t="inlineStr">
+        <is>
+          <t>https://imbue.com/blog/2024-05-09-podcast-episode-35-percy-liang</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="45" t="inlineStr">
+        <is>
+          <t>Konstantine Buhler</t>
+        </is>
+      </c>
+      <c r="B31" s="50" t="inlineStr">
+        <is>
+          <t>Essay</t>
+        </is>
+      </c>
+      <c r="C31" s="46" t="inlineStr">
+        <is>
+          <t>AI Ascent 2025: The Agent Economy (keynote)</t>
+        </is>
+      </c>
+      <c r="D31" s="46" t="inlineStr">
+        <is>
+          <t>Sequoia Capital</t>
+        </is>
+      </c>
+      <c r="E31" s="46" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F31" s="47" t="inlineStr">
+        <is>
+          <t>https://www.sequoiacap.com/article/ai-ascent-2025/</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="40" t="inlineStr">
+        <is>
+          <t>Sonya Huang</t>
+        </is>
+      </c>
+      <c r="B32" s="50" t="inlineStr">
+        <is>
+          <t>Essay</t>
+        </is>
+      </c>
+      <c r="C32" s="42" t="inlineStr">
+        <is>
+          <t>Generative AI's Act o1: The Reasoning Era Begins</t>
+        </is>
+      </c>
+      <c r="D32" s="42" t="inlineStr">
+        <is>
+          <t>Sequoia Capital</t>
+        </is>
+      </c>
+      <c r="E32" s="42" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F32" s="43" t="inlineStr">
+        <is>
+          <t>https://www.sequoiacap.com/article/generative-ais-act-o1/</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="40" t="inlineStr">
+        <is>
+          <t>Sonya Huang</t>
+        </is>
+      </c>
+      <c r="B33" s="50" t="inlineStr">
+        <is>
+          <t>Essay</t>
+        </is>
+      </c>
+      <c r="C33" s="42" t="inlineStr">
+        <is>
+          <t>Generative AI's Act Two</t>
+        </is>
+      </c>
+      <c r="D33" s="42" t="inlineStr">
+        <is>
+          <t>Sequoia Capital</t>
+        </is>
+      </c>
+      <c r="E33" s="42" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="F33" s="43" t="inlineStr">
+        <is>
+          <t>https://www.sequoiacap.com/article/generative-ai-act-two/</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="45" t="inlineStr">
+        <is>
+          <t>Pat Grady</t>
+        </is>
+      </c>
+      <c r="B34" s="44" t="inlineStr">
+        <is>
+          <t>Podcast</t>
+        </is>
+      </c>
+      <c r="C34" s="46" t="inlineStr">
+        <is>
+          <t>Training Data (host; Sequoia AI podcast)</t>
+        </is>
+      </c>
+      <c r="D34" s="46" t="inlineStr">
+        <is>
+          <t>Sequoia Capital</t>
+        </is>
+      </c>
+      <c r="E34" s="46" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F34" s="47" t="inlineStr">
+        <is>
+          <t>https://www.sequoiacap.com/series/training-data/</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="40" t="inlineStr">
+        <is>
+          <t>Martin Casado</t>
+        </is>
+      </c>
+      <c r="B35" s="50" t="inlineStr">
+        <is>
+          <t>Essay</t>
+        </is>
+      </c>
+      <c r="C35" s="42" t="inlineStr">
+        <is>
+          <t>Bitter Economics</t>
+        </is>
+      </c>
+      <c r="D35" s="42" t="inlineStr">
+        <is>
+          <t>a16z</t>
+        </is>
+      </c>
+      <c r="E35" s="42" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F35" s="43" t="inlineStr">
+        <is>
+          <t>https://a16z.com/bitter-economics/</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="40" t="inlineStr">
+        <is>
+          <t>Martin Casado</t>
+        </is>
+      </c>
+      <c r="B36" s="44" t="inlineStr">
+        <is>
+          <t>Podcast</t>
+        </is>
+      </c>
+      <c r="C36" s="42" t="inlineStr">
+        <is>
+          <t>Martin Casado on the Demand Forces Behind AI</t>
+        </is>
+      </c>
+      <c r="D36" s="42" t="inlineStr">
+        <is>
+          <t>AI + a16z</t>
+        </is>
+      </c>
+      <c r="E36" s="42" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F36" s="43" t="inlineStr">
+        <is>
+          <t>https://a16z.com/podcast/martin-casado-on-the-demand-forces-behind-ai/</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="45" t="inlineStr">
+        <is>
+          <t>Anjney Midha</t>
+        </is>
+      </c>
+      <c r="B37" s="50" t="inlineStr">
+        <is>
+          <t>Essay</t>
+        </is>
+      </c>
+      <c r="C37" s="46" t="inlineStr">
+        <is>
+          <t>State of AI: 100 Trillion Token Study with OpenRouter</t>
+        </is>
+      </c>
+      <c r="D37" s="46" t="inlineStr">
+        <is>
+          <t>a16z</t>
+        </is>
+      </c>
+      <c r="E37" s="46" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F37" s="47" t="inlineStr">
+        <is>
+          <t>https://a16z.com/state-of-ai/</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="40" t="inlineStr">
+        <is>
+          <t>Sarah Guo</t>
+        </is>
+      </c>
+      <c r="B38" s="44" t="inlineStr">
+        <is>
+          <t>Podcast</t>
+        </is>
+      </c>
+      <c r="C38" s="42" t="inlineStr">
+        <is>
+          <t>No Priors (co-host w/ Elad Gil)</t>
+        </is>
+      </c>
+      <c r="D38" s="42" t="inlineStr">
+        <is>
+          <t>No Priors</t>
+        </is>
+      </c>
+      <c r="E38" s="42" t="inlineStr">
+        <is>
+          <t>2023-</t>
+        </is>
+      </c>
+      <c r="F38" s="43" t="inlineStr">
+        <is>
+          <t>https://podcasts.apple.com/us/podcast/no-priors-artificial-intelligence-technology-startups/id1668002688</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="40" t="inlineStr">
+        <is>
+          <t>Sarah Guo</t>
+        </is>
+      </c>
+      <c r="B39" s="48" t="inlineStr">
+        <is>
+          <t>Press</t>
+        </is>
+      </c>
+      <c r="C39" s="42" t="inlineStr">
+        <is>
+          <t>Sarah Guo Bet Everything On AI Pre-ChatGPT</t>
+        </is>
+      </c>
+      <c r="D39" s="42" t="inlineStr">
+        <is>
+          <t>Forbes</t>
+        </is>
+      </c>
+      <c r="E39" s="42" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F39" s="43" t="inlineStr">
+        <is>
+          <t>https://www.forbes.com/sites/rashishrivastava/2026/05/27/sarah-guo-bet-everything-on-ai-pre-chatgpt-now-shes-one-of-the-worlds-top-investors/</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="45" t="inlineStr">
+        <is>
+          <t>Elad Gil</t>
+        </is>
+      </c>
+      <c r="B40" s="50" t="inlineStr">
+        <is>
+          <t>Essay</t>
+        </is>
+      </c>
+      <c r="C40" s="46" t="inlineStr">
+        <is>
+          <t>AI Market Clarity</t>
+        </is>
+      </c>
+      <c r="D40" s="46" t="inlineStr">
+        <is>
+          <t>Elad Gil Blog</t>
+        </is>
+      </c>
+      <c r="E40" s="46" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F40" s="47" t="inlineStr">
+        <is>
+          <t>https://blog.eladgil.com/p/ai-market-clarity</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="45" t="inlineStr">
+        <is>
+          <t>Elad Gil</t>
+        </is>
+      </c>
+      <c r="B41" s="48" t="inlineStr">
+        <is>
+          <t>Press</t>
+        </is>
+      </c>
+      <c r="C41" s="46" t="inlineStr">
+        <is>
+          <t>Elad Gil on which AI markets have winners</t>
+        </is>
+      </c>
+      <c r="D41" s="46" t="inlineStr">
+        <is>
+          <t>TechCrunch</t>
+        </is>
+      </c>
+      <c r="E41" s="46" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F41" s="47" t="inlineStr">
+        <is>
+          <t>https://techcrunch.com/2025/11/03/elad-gil-on-which-ai-markets-have-winners-and-which-are-still-wide-open/</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="40" t="inlineStr">
+        <is>
+          <t>Nathan Benaich</t>
+        </is>
+      </c>
+      <c r="B42" s="50" t="inlineStr">
+        <is>
+          <t>Essay</t>
+        </is>
+      </c>
+      <c r="C42" s="42" t="inlineStr">
+        <is>
+          <t>State of AI Report 2025</t>
+        </is>
+      </c>
+      <c r="D42" s="42" t="inlineStr">
+        <is>
+          <t>stateof.ai</t>
+        </is>
+      </c>
+      <c r="E42" s="42" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F42" s="43" t="inlineStr">
+        <is>
+          <t>https://www.stateof.ai/</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="40" t="inlineStr">
+        <is>
+          <t>Nathan Benaich</t>
+        </is>
+      </c>
+      <c r="B43" s="44" t="inlineStr">
+        <is>
+          <t>Podcast</t>
+        </is>
+      </c>
+      <c r="C43" s="42" t="inlineStr">
+        <is>
+          <t>Investing on the Front Lines of the AI Arms Race</t>
+        </is>
+      </c>
+      <c r="D43" s="42" t="inlineStr">
+        <is>
+          <t>Hidden Forces</t>
+        </is>
+      </c>
+      <c r="E43" s="42" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F43" s="43" t="inlineStr">
+        <is>
+          <t>https://hiddenforces.io/podcasts/investing-on-the-front-lines-of-the-ai-arms-race-nathan-benaich/</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="45" t="inlineStr">
+        <is>
+          <t>Matt Turck</t>
+        </is>
+      </c>
+      <c r="B44" s="50" t="inlineStr">
+        <is>
+          <t>Essay</t>
+        </is>
+      </c>
+      <c r="C44" s="46" t="inlineStr">
+        <is>
+          <t>Bubble and Build: The 2025 MAD Landscape</t>
+        </is>
+      </c>
+      <c r="D44" s="46" t="inlineStr">
+        <is>
+          <t>FirstMark</t>
+        </is>
+      </c>
+      <c r="E44" s="46" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F44" s="47" t="inlineStr">
+        <is>
+          <t>https://firstmark.com/story/bubble-build-the-2025-mad-machine-learning-ai-data-landscape/</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="45" t="inlineStr">
+        <is>
+          <t>Matt Turck</t>
+        </is>
+      </c>
+      <c r="B45" s="50" t="inlineStr">
+        <is>
+          <t>Essay</t>
+        </is>
+      </c>
+      <c r="C45" s="46" t="inlineStr">
+        <is>
+          <t>2025 MAD Landscape (interactive)</t>
+        </is>
+      </c>
+      <c r="D45" s="46" t="inlineStr">
+        <is>
+          <t>mad.firstmark.com</t>
+        </is>
+      </c>
+      <c r="E45" s="46" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F45" s="47" t="inlineStr">
+        <is>
+          <t>https://mad.firstmark.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="40" t="inlineStr">
+        <is>
+          <t>Sarah Tavel</t>
+        </is>
+      </c>
+      <c r="B46" s="44" t="inlineStr">
+        <is>
+          <t>Podcast</t>
+        </is>
+      </c>
+      <c r="C46" s="42" t="inlineStr">
+        <is>
+          <t>20VC: The Future of AI is Selling the Work Not the Tools</t>
+        </is>
+      </c>
+      <c r="D46" s="42" t="inlineStr">
+        <is>
+          <t>20VC</t>
+        </is>
+      </c>
+      <c r="E46" s="42" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F46" s="43" t="inlineStr">
+        <is>
+          <t>https://www.thetwentyminutevc.com/sarah-tavel</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="45" t="inlineStr">
+        <is>
+          <t>Harrison Chase</t>
+        </is>
+      </c>
+      <c r="B47" s="50" t="inlineStr">
+        <is>
+          <t>Essay</t>
+        </is>
+      </c>
+      <c r="C47" s="46" t="inlineStr">
+        <is>
+          <t>The rise of "context engineering"</t>
+        </is>
+      </c>
+      <c r="D47" s="46" t="inlineStr">
+        <is>
+          <t>LangChain Blog</t>
+        </is>
+      </c>
+      <c r="E47" s="46" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F47" s="47" t="inlineStr">
+        <is>
+          <t>https://www.langchain.com/blog/the-rise-of-context-engineering</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="45" t="inlineStr">
+        <is>
+          <t>Harrison Chase</t>
+        </is>
+      </c>
+      <c r="B48" s="44" t="inlineStr">
+        <is>
+          <t>Podcast</t>
+        </is>
+      </c>
+      <c r="C48" s="46" t="inlineStr">
+        <is>
+          <t>Context Engineering Our Way to Long-Horizon Agents</t>
+        </is>
+      </c>
+      <c r="D48" s="46" t="inlineStr">
+        <is>
+          <t>Sequoia Training Data</t>
+        </is>
+      </c>
+      <c r="E48" s="46" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F48" s="47" t="inlineStr">
+        <is>
+          <t>https://www.sequoiacap.com/podcast/context-engineering-our-way-to-long-horizon-agents-langchains-harrison-chase/</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="40" t="inlineStr">
+        <is>
+          <t>Jerry Liu</t>
+        </is>
+      </c>
+      <c r="B49" s="44" t="inlineStr">
+        <is>
+          <t>Podcast</t>
+        </is>
+      </c>
+      <c r="C49" s="42" t="inlineStr">
+        <is>
+          <t>RAG Is A Hack — Jerry Liu of LlamaIndex</t>
+        </is>
+      </c>
+      <c r="D49" s="42" t="inlineStr">
+        <is>
+          <t>Latent Space</t>
+        </is>
+      </c>
+      <c r="E49" s="42" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="F49" s="43" t="inlineStr">
+        <is>
+          <t>https://www.latent.space/p/llamaindex</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="45" t="inlineStr">
+        <is>
+          <t>João Moura</t>
+        </is>
+      </c>
+      <c r="B50" s="48" t="inlineStr">
+        <is>
+          <t>Press</t>
+        </is>
+      </c>
+      <c r="C50" s="46" t="inlineStr">
+        <is>
+          <t>CrewAI uses third-party models to automate business tasks</t>
+        </is>
+      </c>
+      <c r="D50" s="46" t="inlineStr">
+        <is>
+          <t>TechCrunch</t>
+        </is>
+      </c>
+      <c r="E50" s="46" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F50" s="47" t="inlineStr">
+        <is>
+          <t>https://techcrunch.com/2024/10/22/crewai-uses-third-party-models-to-automate-business-tasks/</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="45" t="inlineStr">
+        <is>
+          <t>João Moura</t>
+        </is>
+      </c>
+      <c r="B51" s="44" t="inlineStr">
+        <is>
+          <t>Podcast</t>
+        </is>
+      </c>
+      <c r="C51" s="46" t="inlineStr">
+        <is>
+          <t>Crew AI with João Moura</t>
+        </is>
+      </c>
+      <c r="D51" s="46" t="inlineStr">
+        <is>
+          <t>Software Engineering Daily</t>
+        </is>
+      </c>
+      <c r="E51" s="46" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F51" s="47" t="inlineStr">
+        <is>
+          <t>https://softwareengineeringdaily.com/2025/06/03/crew-ai-with-joao-moura/</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="40" t="inlineStr">
+        <is>
+          <t>Toran Bruce Richards</t>
+        </is>
+      </c>
+      <c r="B52" s="48" t="inlineStr">
+        <is>
+          <t>Press</t>
+        </is>
+      </c>
+      <c r="C52" s="42" t="inlineStr">
+        <is>
+          <t>Fireside Chat: Toran Bruce Richards, Founder, AutoGPT</t>
+        </is>
+      </c>
+      <c r="D52" s="42" t="inlineStr">
+        <is>
+          <t>OpenUK</t>
+        </is>
+      </c>
+      <c r="E52" s="42" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F52" s="43" t="inlineStr">
+        <is>
+          <t>https://openuk.uk/thought-leadership/fireside-chat-toran-bruce-richards-2024-phase-one/</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="45" t="inlineStr">
+        <is>
+          <t>Yohei Nakajima</t>
+        </is>
+      </c>
+      <c r="B53" s="51" t="inlineStr">
+        <is>
+          <t>Repo</t>
+        </is>
+      </c>
+      <c r="C53" s="46" t="inlineStr">
+        <is>
+          <t>babyagi (original task-driven autonomous agent)</t>
+        </is>
+      </c>
+      <c r="D53" s="46" t="inlineStr">
+        <is>
+          <t>GitHub</t>
+        </is>
+      </c>
+      <c r="E53" s="46" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="F53" s="47" t="inlineStr">
+        <is>
+          <t>https://github.com/yoheinakajima/babyagi</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="40" t="inlineStr">
+        <is>
+          <t>Killian Lucas</t>
+        </is>
+      </c>
+      <c r="B54" s="44" t="inlineStr">
+        <is>
+          <t>Podcast</t>
+        </is>
+      </c>
+      <c r="C54" s="42" t="inlineStr">
+        <is>
+          <t>Special interview with Killian Lucas, Author of Open Interpreter</t>
+        </is>
+      </c>
+      <c r="D54" s="42" t="inlineStr">
+        <is>
+          <t>ThursdAI</t>
+        </is>
+      </c>
+      <c r="E54" s="42" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="F54" s="43" t="inlineStr">
+        <is>
+          <t>https://sub.thursdai.news/p/thursdai-special-interview-with-killian</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="45" t="inlineStr">
+        <is>
+          <t>Flo Crivello</t>
+        </is>
+      </c>
+      <c r="B55" s="48" t="inlineStr">
+        <is>
+          <t>Press</t>
+        </is>
+      </c>
+      <c r="C55" s="46" t="inlineStr">
+        <is>
+          <t>This founder had to train his AI not to Rickroll people</t>
+        </is>
+      </c>
+      <c r="D55" s="46" t="inlineStr">
+        <is>
+          <t>TechCrunch</t>
+        </is>
+      </c>
+      <c r="E55" s="46" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F55" s="47" t="inlineStr">
+        <is>
+          <t>https://techcrunch.com/2024/08/21/this-founder-had-to-train-his-ai-to-not-rickroll-people/</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="45" t="inlineStr">
+        <is>
+          <t>Flo Crivello</t>
+        </is>
+      </c>
+      <c r="B56" s="44" t="inlineStr">
+        <is>
+          <t>Podcast</t>
+        </is>
+      </c>
+      <c r="C56" s="46" t="inlineStr">
+        <is>
+          <t>The AI Assistant Revolution with Flo Crivello of Lindy</t>
+        </is>
+      </c>
+      <c r="D56" s="46" t="inlineStr">
+        <is>
+          <t>Cognitive Revolution</t>
+        </is>
+      </c>
+      <c r="E56" s="46" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F56" s="47" t="inlineStr">
+        <is>
+          <t>https://www.cognitiverevolution.ai/the-ai-assistant-revolution-with-flo-crivello-of-lindy-ai/</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="40" t="inlineStr">
+        <is>
+          <t>Div Garg</t>
+        </is>
+      </c>
+      <c r="B57" s="44" t="inlineStr">
+        <is>
+          <t>Podcast</t>
+        </is>
+      </c>
+      <c r="C57" s="42" t="inlineStr">
+        <is>
+          <t>The AI Copilot Revolution with Div Garg of MultiOn</t>
+        </is>
+      </c>
+      <c r="D57" s="42" t="inlineStr">
+        <is>
+          <t>Cognitive Revolution</t>
+        </is>
+      </c>
+      <c r="E57" s="42" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F57" s="43" t="inlineStr">
+        <is>
+          <t>https://www.cognitiverevolution.ai/the-ai-copilot-revolution-with-div-garg-of-multi-on/</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="45" t="inlineStr">
+        <is>
+          <t>Shaw Walters</t>
+        </is>
+      </c>
+      <c r="B58" s="44" t="inlineStr">
+        <is>
+          <t>Podcast</t>
+        </is>
+      </c>
+      <c r="C58" s="46" t="inlineStr">
+        <is>
+          <t>The AI-Crypto Convergence: AI Agents with ai16z's Shaw</t>
+        </is>
+      </c>
+      <c r="D58" s="46" t="inlineStr">
+        <is>
+          <t>Bankless</t>
+        </is>
+      </c>
+      <c r="E58" s="46" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F58" s="47" t="inlineStr">
+        <is>
+          <t>https://www.bankless.com/podcast/the-ai-crypto-convergence-exploring-the-ai-agents-with-ai16zs-shaw</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="40" t="inlineStr">
+        <is>
+          <t>Graham Neubig</t>
+        </is>
+      </c>
+      <c r="B59" s="49" t="inlineStr">
+        <is>
+          <t>Video</t>
+        </is>
+      </c>
+      <c r="C59" s="42" t="inlineStr">
+        <is>
+          <t>Best of 2024 in Agents (Graham Neubig, OpenHands)</t>
+        </is>
+      </c>
+      <c r="D59" s="42" t="inlineStr">
+        <is>
+          <t>Latent Space (YouTube)</t>
+        </is>
+      </c>
+      <c r="E59" s="42" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F59" s="43" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=B6PKVZq2qqo</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="45" t="inlineStr">
+        <is>
+          <t>Dharmesh Shah</t>
+        </is>
+      </c>
+      <c r="B60" s="50" t="inlineStr">
+        <is>
+          <t>Essay</t>
+        </is>
+      </c>
+      <c r="C60" s="46" t="inlineStr">
+        <is>
+          <t>Why The Future Of AI Is Agents</t>
+        </is>
+      </c>
+      <c r="D60" s="46" t="inlineStr">
+        <is>
+          <t>Simple.ai</t>
+        </is>
+      </c>
+      <c r="E60" s="46" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F60" s="47" t="inlineStr">
+        <is>
+          <t>https://simple.ai/p/why-the-future-of-ai-is-agents</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="45" t="inlineStr">
+        <is>
+          <t>Dharmesh Shah</t>
+        </is>
+      </c>
+      <c r="B61" s="44" t="inlineStr">
+        <is>
+          <t>Podcast</t>
+        </is>
+      </c>
+      <c r="C61" s="46" t="inlineStr">
+        <is>
+          <t>The Agent Network — Dharmesh Shah</t>
+        </is>
+      </c>
+      <c r="D61" s="46" t="inlineStr">
+        <is>
+          <t>Latent Space</t>
+        </is>
+      </c>
+      <c r="E61" s="46" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F61" s="47" t="inlineStr">
+        <is>
+          <t>https://www.latent.space/p/dharmesh</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="40" t="inlineStr">
+        <is>
+          <t>Matt Shumer</t>
+        </is>
+      </c>
+      <c r="B62" s="48" t="inlineStr">
+        <is>
+          <t>Press</t>
+        </is>
+      </c>
+      <c r="C62" s="42" t="inlineStr">
+        <is>
+          <t>HyperWrite's Reflection 70B open-source model</t>
+        </is>
+      </c>
+      <c r="D62" s="42" t="inlineStr">
+        <is>
+          <t>VentureBeat</t>
+        </is>
+      </c>
+      <c r="E62" s="42" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F62" s="43" t="inlineStr">
+        <is>
+          <t>https://venturebeat.com/ai/meet-the-new-most-powerful-open-source-ai-model-in-the-world-hyperwrites-reflection-70b</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="45" t="inlineStr">
+        <is>
+          <t>Bret Taylor</t>
+        </is>
+      </c>
+      <c r="B63" s="48" t="inlineStr">
+        <is>
+          <t>Press</t>
+        </is>
+      </c>
+      <c r="C63" s="46" t="inlineStr">
+        <is>
+          <t>Interview with Sierra CEO Bret Taylor about AI Agents</t>
+        </is>
+      </c>
+      <c r="D63" s="46" t="inlineStr">
+        <is>
+          <t>Stratechery</t>
+        </is>
+      </c>
+      <c r="E63" s="46" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F63" s="47" t="inlineStr">
+        <is>
+          <t>https://stratechery.com/2025/an-interview-with-sierra-founder-and-ceo-bret-taylor-about-ai-agents-and-tech-history-lessons/</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="40" t="inlineStr">
+        <is>
+          <t>Scott Wu</t>
+        </is>
+      </c>
+      <c r="B64" s="48" t="inlineStr">
+        <is>
+          <t>Press</t>
+        </is>
+      </c>
+      <c r="C64" s="42" t="inlineStr">
+        <is>
+          <t>Cognition's Scott Wu says AI coding agents shouldn't replace humans</t>
+        </is>
+      </c>
+      <c r="D64" s="42" t="inlineStr">
+        <is>
+          <t>TechCrunch</t>
+        </is>
+      </c>
+      <c r="E64" s="42" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F64" s="43" t="inlineStr">
+        <is>
+          <t>https://techcrunch.com/2026/05/29/cognitions-scott-wu-says-ai-coding-agents-shouldnt-replace-humans/</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="45" t="inlineStr">
+        <is>
+          <t>Kanjun Qiu</t>
+        </is>
+      </c>
+      <c r="B65" s="44" t="inlineStr">
+        <is>
+          <t>Podcast</t>
+        </is>
+      </c>
+      <c r="C65" s="46" t="inlineStr">
+        <is>
+          <t>Why AI Agents Don't Work (yet) — Kanjun Qiu of Imbue</t>
+        </is>
+      </c>
+      <c r="D65" s="46" t="inlineStr">
+        <is>
+          <t>Latent Space</t>
+        </is>
+      </c>
+      <c r="E65" s="46" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="F65" s="47" t="inlineStr">
+        <is>
+          <t>https://www.latent.space/p/imbue</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="40" t="inlineStr">
+        <is>
+          <t>David Luan</t>
+        </is>
+      </c>
+      <c r="B66" s="48" t="inlineStr">
+        <is>
+          <t>Press</t>
+        </is>
+      </c>
+      <c r="C66" s="42" t="inlineStr">
+        <is>
+          <t>Amazon AGI Labs chief defends his reverse acqui-hire</t>
+        </is>
+      </c>
+      <c r="D66" s="42" t="inlineStr">
+        <is>
+          <t>TechCrunch</t>
+        </is>
+      </c>
+      <c r="E66" s="42" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F66" s="43" t="inlineStr">
+        <is>
+          <t>https://techcrunch.com/2025/08/23/amazon-agi-labs-chief-defends-his-reverse-acquihire/</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="45" t="inlineStr">
+        <is>
+          <t>Aravind Srinivas</t>
+        </is>
+      </c>
+      <c r="B67" s="48" t="inlineStr">
+        <is>
+          <t>Press</t>
+        </is>
+      </c>
+      <c r="C67" s="46" t="inlineStr">
+        <is>
+          <t>Aravind Srinivas on the Infinite Value of Knowledge</t>
+        </is>
+      </c>
+      <c r="D67" s="46" t="inlineStr">
+        <is>
+          <t>Stanford GSB</t>
+        </is>
+      </c>
+      <c r="E67" s="46" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F67" s="47" t="inlineStr">
+        <is>
+          <t>https://www.gsb.stanford.edu/insights/perplexitys-aravind-srinivas-infinite-value-knowledge</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="40" t="inlineStr">
+        <is>
+          <t>Jesse Zhang</t>
+        </is>
+      </c>
+      <c r="B68" s="44" t="inlineStr">
+        <is>
+          <t>Podcast</t>
+        </is>
+      </c>
+      <c r="C68" s="42" t="inlineStr">
+        <is>
+          <t>Decagon's Jesse Zhang: To Win in Agentic AI, Focus on Your Customer</t>
+        </is>
+      </c>
+      <c r="D68" s="42" t="inlineStr">
+        <is>
+          <t>Accel</t>
+        </is>
+      </c>
+      <c r="E68" s="42" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F68" s="43" t="inlineStr">
+        <is>
+          <t>https://www.accel.com/podcast-episodes/decagons-jesse-zhang-to-win-in-agentic-ai-focus-on-your-customer</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="45" t="inlineStr">
+        <is>
+          <t>Winston Weinberg</t>
+        </is>
+      </c>
+      <c r="B69" s="48" t="inlineStr">
+        <is>
+          <t>Press</t>
+        </is>
+      </c>
+      <c r="C69" s="46" t="inlineStr">
+        <is>
+          <t>Inside Harvey: how a first-year associate built a hot startup</t>
+        </is>
+      </c>
+      <c r="D69" s="46" t="inlineStr">
+        <is>
+          <t>TechCrunch</t>
+        </is>
+      </c>
+      <c r="E69" s="46" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F69" s="47" t="inlineStr">
+        <is>
+          <t>https://techcrunch.com/2025/11/14/inside-harvey-how-a-first-year-legal-associate-built-one-of-silicon-valleys-hottest-startups/</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="40" t="inlineStr">
+        <is>
+          <t>Jaspar Carmichael-Jack</t>
+        </is>
+      </c>
+      <c r="B70" s="48" t="inlineStr">
+        <is>
+          <t>Press</t>
+        </is>
+      </c>
+      <c r="C70" s="42" t="inlineStr">
+        <is>
+          <t>Stop hiring the wrong humans, Artisan's founder says</t>
+        </is>
+      </c>
+      <c r="D70" s="42" t="inlineStr">
+        <is>
+          <t>TechCrunch</t>
+        </is>
+      </c>
+      <c r="E70" s="42" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F70" s="43" t="inlineStr">
+        <is>
+          <t>https://techcrunch.com/2026/04/23/dont-stop-hiring-humans-stop-hiring-the-wrong-humans-artisans-founder-says/</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="45" t="inlineStr">
+        <is>
+          <t>Matan Grinberg</t>
+        </is>
+      </c>
+      <c r="B71" s="44" t="inlineStr">
+        <is>
+          <t>Podcast</t>
+        </is>
+      </c>
+      <c r="C71" s="46" t="inlineStr">
+        <is>
+          <t>Factory Unleashes the Droids on Software Development</t>
+        </is>
+      </c>
+      <c r="D71" s="46" t="inlineStr">
+        <is>
+          <t>Sequoia Training Data</t>
+        </is>
+      </c>
+      <c r="E71" s="46" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F71" s="47" t="inlineStr">
+        <is>
+          <t>https://sequoiacap.com/podcast/training-data-factory/</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="40" t="inlineStr">
+        <is>
+          <t>Noam Shazeer</t>
+        </is>
+      </c>
+      <c r="B72" s="48" t="inlineStr">
+        <is>
+          <t>Press</t>
+        </is>
+      </c>
+      <c r="C72" s="42" t="inlineStr">
+        <is>
+          <t>Character.AI's Noam Shazeer on what we know about AI</t>
+        </is>
+      </c>
+      <c r="D72" s="42" t="inlineStr">
+        <is>
+          <t>Fortune</t>
+        </is>
+      </c>
+      <c r="E72" s="42" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F72" s="43" t="inlineStr">
+        <is>
+          <t>https://fortune.com/2024/08/02/character-ais-noam-shazeer-what-we-know-about-ai/</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="45" t="inlineStr">
+        <is>
+          <t>Mustafa Suleyman</t>
+        </is>
+      </c>
+      <c r="B73" s="50" t="inlineStr">
+        <is>
+          <t>Essay</t>
+        </is>
+      </c>
+      <c r="C73" s="46" t="inlineStr">
+        <is>
+          <t>Seemingly Conscious AI is Coming</t>
+        </is>
+      </c>
+      <c r="D73" s="46" t="inlineStr">
+        <is>
+          <t>mustafa-suleyman.ai</t>
+        </is>
+      </c>
+      <c r="E73" s="46" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F73" s="47" t="inlineStr">
+        <is>
+          <t>https://mustafa-suleyman.ai/seemingly-conscious-ai-is-coming</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="40" t="inlineStr">
+        <is>
+          <t>Charles Lamanna</t>
+        </is>
+      </c>
+      <c r="B74" s="48" t="inlineStr">
+        <is>
+          <t>Press</t>
+        </is>
+      </c>
+      <c r="C74" s="42" t="inlineStr">
+        <is>
+          <t>AI Agents and Copilots 'Completely Change' How We Work</t>
+        </is>
+      </c>
+      <c r="D74" s="42" t="inlineStr">
+        <is>
+          <t>Cloud Wars</t>
+        </is>
+      </c>
+      <c r="E74" s="42" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F74" s="43" t="inlineStr">
+        <is>
+          <t>https://cloudwars.com/ai/charles-lamanna-of-microsoft-ai-agents-and-copilots-completely-change-how-we-work/</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="45" t="inlineStr">
+        <is>
+          <t>Kevin Weil</t>
+        </is>
+      </c>
+      <c r="B75" s="44" t="inlineStr">
+        <is>
+          <t>Podcast</t>
+        </is>
+      </c>
+      <c r="C75" s="46" t="inlineStr">
+        <is>
+          <t>OpenAI's CPO on how AI changes must-have skills, moats, coding</t>
+        </is>
+      </c>
+      <c r="D75" s="46" t="inlineStr">
+        <is>
+          <t>Lenny's Podcast</t>
+        </is>
+      </c>
+      <c r="E75" s="46" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F75" s="47" t="inlineStr">
+        <is>
+          <t>https://www.lennysnewsletter.com/p/kevin-weil-open-ai</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="40" t="inlineStr">
+        <is>
+          <t>Marc Benioff</t>
+        </is>
+      </c>
+      <c r="B76" s="48" t="inlineStr">
+        <is>
+          <t>Press</t>
+        </is>
+      </c>
+      <c r="C76" s="42" t="inlineStr">
+        <is>
+          <t>Interview with Salesforce CEO Marc Benioff about AI Abundance</t>
+        </is>
+      </c>
+      <c r="D76" s="42" t="inlineStr">
+        <is>
+          <t>Stratechery</t>
+        </is>
+      </c>
+      <c r="E76" s="42" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F76" s="43" t="inlineStr">
+        <is>
+          <t>https://stratechery.com/2024/an-interview-with-salesforce-ceo-marc-benioff-about-ai-abundance/</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="45" t="inlineStr">
+        <is>
+          <t>Josh Woodward</t>
+        </is>
+      </c>
+      <c r="B77" s="44" t="inlineStr">
+        <is>
+          <t>Podcast</t>
+        </is>
+      </c>
+      <c r="C77" s="46" t="inlineStr">
+        <is>
+          <t>How Google Labs is Pushing the Frontier of AI Applications</t>
+        </is>
+      </c>
+      <c r="D77" s="46" t="inlineStr">
+        <is>
+          <t>Sequoia Training Data</t>
+        </is>
+      </c>
+      <c r="E77" s="46" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F77" s="47" t="inlineStr">
+        <is>
+          <t>https://sequoiacap.com/podcast/training-data-josh-woodward/</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="40" t="inlineStr">
+        <is>
+          <t>Xiao Hong (肖弘) &amp; Ji Yichao (季逸超)</t>
+        </is>
+      </c>
+      <c r="B78" s="48" t="inlineStr">
+        <is>
+          <t>Press</t>
+        </is>
+      </c>
+      <c r="C78" s="42" t="inlineStr">
+        <is>
+          <t>Manus Xiao Hong: The Caulker of Idealism</t>
+        </is>
+      </c>
+      <c r="D78" s="42" t="inlineStr">
+        <is>
+          <t>36Kr (EN)</t>
+        </is>
+      </c>
+      <c r="E78" s="42" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F78" s="43" t="inlineStr">
+        <is>
+          <t>https://eu.36kr.com/en/p/3707111546712197</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="40" t="inlineStr">
+        <is>
+          <t>Xiao Hong (肖弘) &amp; Ji Yichao (季逸超)</t>
+        </is>
+      </c>
+      <c r="B79" s="48" t="inlineStr">
+        <is>
+          <t>Press</t>
+        </is>
+      </c>
+      <c r="C79" s="42" t="inlineStr">
+        <is>
+          <t>How Yichao "Peak" Ji became a global AI app hitmaker</t>
+        </is>
+      </c>
+      <c r="D79" s="42" t="inlineStr">
+        <is>
+          <t>MIT Technology Review</t>
+        </is>
+      </c>
+      <c r="E79" s="42" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F79" s="43" t="inlineStr">
+        <is>
+          <t>https://www.technologyreview.com/2025/09/08/1122642/ji-peak-yichao-innovator-manus-app-ai/</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="45" t="inlineStr">
+        <is>
+          <t>Tang Jie (唐杰)</t>
+        </is>
+      </c>
+      <c r="B80" s="41" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C80" s="46" t="inlineStr">
+        <is>
+          <t>AgentBench: Evaluating LLMs as Agents</t>
+        </is>
+      </c>
+      <c r="D80" s="46" t="inlineStr">
+        <is>
+          <t>arXiv (ICLR 2024)</t>
+        </is>
+      </c>
+      <c r="E80" s="46" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="F80" s="47" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2308.03688</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="45" t="inlineStr">
+        <is>
+          <t>Tang Jie (唐杰)</t>
+        </is>
+      </c>
+      <c r="B81" s="41" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C81" s="46" t="inlineStr">
+        <is>
+          <t>AutoGLM: Autonomous Foundation Agents for GUIs</t>
+        </is>
+      </c>
+      <c r="D81" s="46" t="inlineStr">
+        <is>
+          <t>arXiv</t>
+        </is>
+      </c>
+      <c r="E81" s="46" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F81" s="47" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2411.00820</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="40" t="inlineStr">
+        <is>
+          <t>Liu Zhiyuan (刘知远)</t>
+        </is>
+      </c>
+      <c r="B82" s="41" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C82" s="42" t="inlineStr">
+        <is>
+          <t>ChatDev: Communicative Agents for Software Development</t>
+        </is>
+      </c>
+      <c r="D82" s="42" t="inlineStr">
+        <is>
+          <t>arXiv (ACL 2024)</t>
+        </is>
+      </c>
+      <c r="E82" s="42" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="F82" s="43" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2307.07924</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="40" t="inlineStr">
+        <is>
+          <t>Liu Zhiyuan (刘知远)</t>
+        </is>
+      </c>
+      <c r="B83" s="49" t="inlineStr">
+        <is>
+          <t>Talk</t>
+        </is>
+      </c>
+      <c r="C83" s="42" t="inlineStr">
+        <is>
+          <t>大模型驱动的自主智能体和群体智能</t>
+        </is>
+      </c>
+      <c r="D83" s="42" t="inlineStr">
+        <is>
+          <t>36Kr WISE2023</t>
+        </is>
+      </c>
+      <c r="E83" s="42" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="F83" s="43" t="inlineStr">
+        <is>
+          <t>https://36kr.com/p/2540349049300481</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="45" t="inlineStr">
+        <is>
+          <t>Yang Zhilin (杨植麟)</t>
+        </is>
+      </c>
+      <c r="B84" s="48" t="inlineStr">
+        <is>
+          <t>Press</t>
+        </is>
+      </c>
+      <c r="C84" s="46" t="inlineStr">
+        <is>
+          <t>100 Hours Inside Moonshot AI</t>
+        </is>
+      </c>
+      <c r="D84" s="46" t="inlineStr">
+        <is>
+          <t>Recode China AI</t>
+        </is>
+      </c>
+      <c r="E84" s="46" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F84" s="47" t="inlineStr">
+        <is>
+          <t>https://www.recodechinaai.com/p/deepseek-and-moonshot-the-ai-labs</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="45" t="inlineStr">
+        <is>
+          <t>Yang Zhilin (杨植麟)</t>
+        </is>
+      </c>
+      <c r="B85" s="41" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C85" s="46" t="inlineStr">
+        <is>
+          <t>XLNet: Generalized Autoregressive Pretraining</t>
+        </is>
+      </c>
+      <c r="D85" s="46" t="inlineStr">
+        <is>
+          <t>arXiv (NeurIPS 2019)</t>
+        </is>
+      </c>
+      <c r="E85" s="46" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="F85" s="47" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/1906.08237</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="40" t="inlineStr">
+        <is>
+          <t>Yan Junjie (闫俊杰)</t>
+        </is>
+      </c>
+      <c r="B86" s="48" t="inlineStr">
+        <is>
+          <t>Press</t>
+        </is>
+      </c>
+      <c r="C86" s="42" t="inlineStr">
+        <is>
+          <t>Four-hour Interview: Yan Junjie of MiniMax &amp; Luo Yonghao</t>
+        </is>
+      </c>
+      <c r="D86" s="42" t="inlineStr">
+        <is>
+          <t>36Kr (EN)</t>
+        </is>
+      </c>
+      <c r="E86" s="42" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F86" s="43" t="inlineStr">
+        <is>
+          <t>https://eu.36kr.com/en/p/3590840490688517</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="45" t="inlineStr">
+        <is>
+          <t>Liang Wenfeng (梁文锋)</t>
+        </is>
+      </c>
+      <c r="B87" s="48" t="inlineStr">
+        <is>
+          <t>Press</t>
+        </is>
+      </c>
+      <c r="C87" s="46" t="inlineStr">
+        <is>
+          <t>DeepSeek: The Quiet Giant Leading China's AI Race</t>
+        </is>
+      </c>
+      <c r="D87" s="46" t="inlineStr">
+        <is>
+          <t>ChinaTalk</t>
+        </is>
+      </c>
+      <c r="E87" s="46" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F87" s="47" t="inlineStr">
+        <is>
+          <t>https://www.chinatalk.media/p/deepseek-ceo-interview-with-chinas</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="45" t="inlineStr">
+        <is>
+          <t>Liang Wenfeng (梁文锋)</t>
+        </is>
+      </c>
+      <c r="B88" s="41" t="inlineStr">
+        <is>
+          <t>Paper</t>
+        </is>
+      </c>
+      <c r="C88" s="46" t="inlineStr">
+        <is>
+          <t>DeepSeek-R1: Incentivizing Reasoning via RL</t>
+        </is>
+      </c>
+      <c r="D88" s="46" t="inlineStr">
+        <is>
+          <t>arXiv</t>
+        </is>
+      </c>
+      <c r="E88" s="46" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F88" s="47" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2501.12948</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="40" t="inlineStr">
+        <is>
+          <t>Zhu Zheqing (朱哲清)</t>
+        </is>
+      </c>
+      <c r="B89" s="49" t="inlineStr">
+        <is>
+          <t>Video</t>
+        </is>
+      </c>
+      <c r="C89" s="42" t="inlineStr">
+        <is>
+          <t>AI Startup CEO Spotlight: Bill Zhu, Pokee AI</t>
+        </is>
+      </c>
+      <c r="D89" s="42" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="E89" s="42" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F89" s="43" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=7ioAxX8khgM</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="45" t="inlineStr">
+        <is>
+          <t>Andrej Karpathy</t>
+        </is>
+      </c>
+      <c r="B90" s="49" t="inlineStr">
+        <is>
+          <t>Video</t>
+        </is>
+      </c>
+      <c r="C90" s="46" t="inlineStr">
+        <is>
+          <t>Software Is Changing (Again) — Software 3.0</t>
+        </is>
+      </c>
+      <c r="D90" s="46" t="inlineStr">
+        <is>
+          <t>Y Combinator</t>
+        </is>
+      </c>
+      <c r="E90" s="46" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F90" s="47" t="inlineStr">
+        <is>
+          <t>https://www.ycombinator.com/library/MW-andrej-karpathy-software-is-changing-again</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="40" t="inlineStr">
+        <is>
+          <t>Swyx (Shawn Wang)</t>
+        </is>
+      </c>
+      <c r="B91" s="50" t="inlineStr">
+        <is>
+          <t>Essay</t>
+        </is>
+      </c>
+      <c r="C91" s="42" t="inlineStr">
+        <is>
+          <t>The Rise of the AI Engineer</t>
+        </is>
+      </c>
+      <c r="D91" s="42" t="inlineStr">
+        <is>
+          <t>Latent Space</t>
+        </is>
+      </c>
+      <c r="E91" s="42" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="F91" s="43" t="inlineStr">
+        <is>
+          <t>https://www.latent.space/p/ai-engineer</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="45" t="inlineStr">
+        <is>
+          <t>Ethan Mollick</t>
+        </is>
+      </c>
+      <c r="B92" s="50" t="inlineStr">
+        <is>
+          <t>Post</t>
+        </is>
+      </c>
+      <c r="C92" s="46" t="inlineStr">
+        <is>
+          <t>Real AI Agents and Real Work</t>
+        </is>
+      </c>
+      <c r="D92" s="46" t="inlineStr">
+        <is>
+          <t>One Useful Thing</t>
+        </is>
+      </c>
+      <c r="E92" s="46" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F92" s="47" t="inlineStr">
+        <is>
+          <t>https://www.oneusefulthing.org/p/real-ai-agents-and-real-work</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="45" t="inlineStr">
+        <is>
+          <t>Ethan Mollick</t>
+        </is>
+      </c>
+      <c r="B93" s="50" t="inlineStr">
+        <is>
+          <t>Post</t>
+        </is>
+      </c>
+      <c r="C93" s="46" t="inlineStr">
+        <is>
+          <t>The Shape of the Thing</t>
+        </is>
+      </c>
+      <c r="D93" s="46" t="inlineStr">
+        <is>
+          <t>One Useful Thing</t>
+        </is>
+      </c>
+      <c r="E93" s="46" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F93" s="47" t="inlineStr">
+        <is>
+          <t>https://www.oneusefulthing.org/p/the-shape-of-the-thing</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="40" t="inlineStr">
+        <is>
+          <t>Simon Willison</t>
+        </is>
+      </c>
+      <c r="B94" s="50" t="inlineStr">
+        <is>
+          <t>Post</t>
+        </is>
+      </c>
+      <c r="C94" s="42" t="inlineStr">
+        <is>
+          <t>Agentic Coding: The Future of Software Development with Agents</t>
+        </is>
+      </c>
+      <c r="D94" s="42" t="inlineStr">
+        <is>
+          <t>simonwillison.net</t>
+        </is>
+      </c>
+      <c r="E94" s="42" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F94" s="43" t="inlineStr">
+        <is>
+          <t>https://simonwillison.net/2025/Jun/29/agentic-coding/</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="40" t="inlineStr">
+        <is>
+          <t>Simon Willison</t>
+        </is>
+      </c>
+      <c r="B95" s="50" t="inlineStr">
+        <is>
+          <t>Post</t>
+        </is>
+      </c>
+      <c r="C95" s="42" t="inlineStr">
+        <is>
+          <t>Code execution with MCP: Building more efficient agents</t>
+        </is>
+      </c>
+      <c r="D95" s="42" t="inlineStr">
+        <is>
+          <t>simonwillison.net</t>
+        </is>
+      </c>
+      <c r="E95" s="42" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F95" s="43" t="inlineStr">
+        <is>
+          <t>https://simonwillison.net/2025/Nov/4/code-execution-with-mcp/</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="45" t="inlineStr">
+        <is>
+          <t>Nathan Lambert</t>
+        </is>
+      </c>
+      <c r="B96" s="50" t="inlineStr">
+        <is>
+          <t>Post</t>
+        </is>
+      </c>
+      <c r="C96" s="46" t="inlineStr">
+        <is>
+          <t>Interconnects (newsletter home)</t>
+        </is>
+      </c>
+      <c r="D96" s="46" t="inlineStr">
+        <is>
+          <t>Substack</t>
+        </is>
+      </c>
+      <c r="E96" s="46" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F96" s="47" t="inlineStr">
+        <is>
+          <t>https://www.interconnects.ai/</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="40" t="inlineStr">
+        <is>
+          <t>Dan Shipper</t>
+        </is>
+      </c>
+      <c r="B97" s="50" t="inlineStr">
+        <is>
+          <t>Post</t>
+        </is>
+      </c>
+      <c r="C97" s="42" t="inlineStr">
+        <is>
+          <t>Chain of Thought (column home)</t>
+        </is>
+      </c>
+      <c r="D97" s="42" t="inlineStr">
+        <is>
+          <t>Every</t>
+        </is>
+      </c>
+      <c r="E97" s="42" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F97" s="43" t="inlineStr">
+        <is>
+          <t>https://every.to/chain-of-thought</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="45" t="inlineStr">
+        <is>
+          <t>Rowan Cheung</t>
+        </is>
+      </c>
+      <c r="B98" s="50" t="inlineStr">
+        <is>
+          <t>Post</t>
+        </is>
+      </c>
+      <c r="C98" s="46" t="inlineStr">
+        <is>
+          <t>The Rundown AI (newsletter home)</t>
+        </is>
+      </c>
+      <c r="D98" s="46" t="inlineStr">
+        <is>
+          <t>The Rundown AI</t>
+        </is>
+      </c>
+      <c r="E98" s="46" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F98" s="47" t="inlineStr">
+        <is>
+          <t>https://www.therundown.ai/</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="40" t="inlineStr">
+        <is>
+          <t>Zvi Mowshowitz</t>
+        </is>
+      </c>
+      <c r="B99" s="50" t="inlineStr">
+        <is>
+          <t>Post</t>
+        </is>
+      </c>
+      <c r="C99" s="42" t="inlineStr">
+        <is>
+          <t>Don't Worry About the Vase (home)</t>
+        </is>
+      </c>
+      <c r="D99" s="42" t="inlineStr">
+        <is>
+          <t>Substack</t>
+        </is>
+      </c>
+      <c r="E99" s="42" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F99" s="43" t="inlineStr">
+        <is>
+          <t>https://thezvi.substack.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="45" t="inlineStr">
+        <is>
+          <t>Stephanie Palazzolo</t>
+        </is>
+      </c>
+      <c r="B100" s="48" t="inlineStr">
+        <is>
+          <t>Press</t>
+        </is>
+      </c>
+      <c r="C100" s="46" t="inlineStr">
+        <is>
+          <t>AI Agenda (newsletter)</t>
+        </is>
+      </c>
+      <c r="D100" s="46" t="inlineStr">
+        <is>
+          <t>The Information</t>
+        </is>
+      </c>
+      <c r="E100" s="46" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F100" s="47" t="inlineStr">
+        <is>
+          <t>https://www.theinformation.com/features/ai-agenda</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="40" t="inlineStr">
+        <is>
+          <t>David Soria Parra &amp; Justin Spahr-Summers</t>
+        </is>
+      </c>
+      <c r="B101" s="50" t="inlineStr">
+        <is>
+          <t>Post</t>
+        </is>
+      </c>
+      <c r="C101" s="42" t="inlineStr">
+        <is>
+          <t>Introducing the Model Context Protocol</t>
+        </is>
+      </c>
+      <c r="D101" s="42" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="E101" s="42" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F101" s="43" t="inlineStr">
+        <is>
+          <t>https://www.anthropic.com/news/model-context-protocol</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="45" t="inlineStr">
+        <is>
+          <t>Sean Neville</t>
+        </is>
+      </c>
+      <c r="B102" s="50" t="inlineStr">
+        <is>
+          <t>Post</t>
+        </is>
+      </c>
+      <c r="C102" s="46" t="inlineStr">
+        <is>
+          <t>Agent Commerce Kit (ACK): Enabling the Agent Economy</t>
+        </is>
+      </c>
+      <c r="D102" s="46" t="inlineStr">
+        <is>
+          <t>Catena Labs</t>
+        </is>
+      </c>
+      <c r="E102" s="46" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F102" s="47" t="inlineStr">
+        <is>
+          <t>https://catena.com/blog/agent-commerce-kit</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="40" t="inlineStr">
+        <is>
+          <t>Amir Sarhangi &amp; Craig DeWitt</t>
+        </is>
+      </c>
+      <c r="B103" s="48" t="inlineStr">
+        <is>
+          <t>Press</t>
+        </is>
+      </c>
+      <c r="C103" s="42" t="inlineStr">
+        <is>
+          <t>Skyfire lets AI agents spend your money</t>
+        </is>
+      </c>
+      <c r="D103" s="42" t="inlineStr">
+        <is>
+          <t>TechCrunch</t>
+        </is>
+      </c>
+      <c r="E103" s="42" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F103" s="43" t="inlineStr">
+        <is>
+          <t>https://techcrunch.com/2024/08/21/skyfire-lets-ai-agents-spend-your-money/</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="45" t="inlineStr">
+        <is>
+          <t>Tyllen Bicakcic</t>
+        </is>
+      </c>
+      <c r="B104" s="50" t="inlineStr">
+        <is>
+          <t>Post</t>
+        </is>
+      </c>
+      <c r="C104" s="46" t="inlineStr">
+        <is>
+          <t>About Us (mission)</t>
+        </is>
+      </c>
+      <c r="D104" s="46" t="inlineStr">
+        <is>
+          <t>Payman AI</t>
+        </is>
+      </c>
+      <c r="E104" s="46" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F104" s="47" t="inlineStr">
+        <is>
+          <t>https://paymanai.com/about-us</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="40" t="inlineStr">
+        <is>
+          <t>Illia Polosukhin</t>
+        </is>
+      </c>
+      <c r="B105" s="49" t="inlineStr">
+        <is>
+          <t>Video</t>
+        </is>
+      </c>
+      <c r="C105" s="42" t="inlineStr">
+        <is>
+          <t>AI should optimize your life — not companies' profits</t>
+        </is>
+      </c>
+      <c r="D105" s="42" t="inlineStr">
+        <is>
+          <t>TED (TEDAI SF)</t>
+        </is>
+      </c>
+      <c r="E105" s="42" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F105" s="43" t="inlineStr">
+        <is>
+          <t>https://www.ted.com/talks/illia_polosukhin_ai_should_optimize_your_life_not_companies_profits</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="45" t="inlineStr">
+        <is>
+          <t>Jansen (Wee Kee) Teng</t>
+        </is>
+      </c>
+      <c r="B106" s="52" t="inlineStr">
+        <is>
+          <t>Whitepaper</t>
+        </is>
+      </c>
+      <c r="C106" s="46" t="inlineStr">
+        <is>
+          <t>Virtuals Protocol Whitepaper</t>
+        </is>
+      </c>
+      <c r="D106" s="46" t="inlineStr">
+        <is>
+          <t>Virtuals</t>
+        </is>
+      </c>
+      <c r="E106" s="46" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F106" s="47" t="inlineStr">
+        <is>
+          <t>https://whitepaper.virtuals.io/</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="45" t="inlineStr">
+        <is>
+          <t>Jansen (Wee Kee) Teng</t>
+        </is>
+      </c>
+      <c r="B107" s="48" t="inlineStr">
+        <is>
+          <t>Press</t>
+        </is>
+      </c>
+      <c r="C107" s="46" t="inlineStr">
+        <is>
+          <t>AI agents are evolving into autonomous economic actors</t>
+        </is>
+      </c>
+      <c r="D107" s="46" t="inlineStr">
+        <is>
+          <t>CoinDesk</t>
+        </is>
+      </c>
+      <c r="E107" s="46" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F107" s="47" t="inlineStr">
+        <is>
+          <t>https://www.coindesk.com/coindesk-news/2026/06/26/virtuals-jansen-teng-says-ai-agents-are-evolving-into-autonomous-economic-actors</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="40" t="inlineStr">
+        <is>
+          <t>Humayun Sheikh</t>
+        </is>
+      </c>
+      <c r="B108" s="50" t="inlineStr">
+        <is>
+          <t>Post</t>
+        </is>
+      </c>
+      <c r="C108" s="42" t="inlineStr">
+        <is>
+          <t>Introducing the Artificial Superintelligence Alliance</t>
+        </is>
+      </c>
+      <c r="D108" s="42" t="inlineStr">
+        <is>
+          <t>SingularityNET</t>
+        </is>
+      </c>
+      <c r="E108" s="42" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F108" s="43" t="inlineStr">
+        <is>
+          <t>https://singularitynet.io/introducing-the-artificial-superintelligence-alliance/</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="45" t="inlineStr">
+        <is>
+          <t>David Minarsch</t>
+        </is>
+      </c>
+      <c r="B109" s="52" t="inlineStr">
+        <is>
+          <t>Whitepaper</t>
+        </is>
+      </c>
+      <c r="C109" s="46" t="inlineStr">
+        <is>
+          <t>Autonolas Whitepaper v1.0</t>
+        </is>
+      </c>
+      <c r="D109" s="46" t="inlineStr">
+        <is>
+          <t>olas.network</t>
+        </is>
+      </c>
+      <c r="E109" s="46" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="F109" s="47" t="inlineStr">
+        <is>
+          <t>https://olas.network/documents/whitepaper/Whitepaper%20v1.0.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="45" t="inlineStr">
+        <is>
+          <t>David Minarsch</t>
+        </is>
+      </c>
+      <c r="B110" s="48" t="inlineStr">
+        <is>
+          <t>Press</t>
+        </is>
+      </c>
+      <c r="C110" s="46" t="inlineStr">
+        <is>
+          <t>Olas raises $13.8M for decentralized app store for AI agents</t>
+        </is>
+      </c>
+      <c r="D110" s="46" t="inlineStr">
+        <is>
+          <t>SiliconANGLE</t>
+        </is>
+      </c>
+      <c r="E110" s="46" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F110" s="47" t="inlineStr">
+        <is>
+          <t>https://siliconangle.com/2025/02/05/olas-raises-13-8m-launch-decentralized-app-store-ai-agents/</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="40" t="inlineStr">
+        <is>
+          <t>Jason Zhao &amp; SY Lee</t>
+        </is>
+      </c>
+      <c r="B111" s="52" t="inlineStr">
+        <is>
+          <t>Whitepaper</t>
+        </is>
+      </c>
+      <c r="C111" s="42" t="inlineStr">
+        <is>
+          <t>Agent TCP/IP: An Agent-to-Agent Transaction System</t>
+        </is>
+      </c>
+      <c r="D111" s="42" t="inlineStr">
+        <is>
+          <t>arXiv (Story)</t>
+        </is>
+      </c>
+      <c r="E111" s="42" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F111" s="43" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/pdf/2501.06243</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="40" t="inlineStr">
+        <is>
+          <t>Jason Zhao &amp; SY Lee</t>
+        </is>
+      </c>
+      <c r="B112" s="48" t="inlineStr">
+        <is>
+          <t>Press</t>
+        </is>
+      </c>
+      <c r="C112" s="42" t="inlineStr">
+        <is>
+          <t>Story raises $80M to build a blockchain for content IP</t>
+        </is>
+      </c>
+      <c r="D112" s="42" t="inlineStr">
+        <is>
+          <t>TechCrunch</t>
+        </is>
+      </c>
+      <c r="E112" s="42" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F112" s="43" t="inlineStr">
+        <is>
+          <t>https://techcrunch.com/2024/08/21/story-raises-83m-at-a-2-25b-valuation-to-build-a-blockchain-for-the-business-of-content-ip-in-the-age-of-ai/</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:F112"/>
+  <mergeCells count="2">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F23" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F26" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F27" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F29" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F30" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F31" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F32" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F33" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F34" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F35" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F36" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F37" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F38" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F39" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F40" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F41" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F42" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F43" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F44" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F45" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F46" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F47" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F48" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F49" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F50" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F51" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F52" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F53" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F54" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F55" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F56" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F57" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F58" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F59" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F60" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F61" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F62" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F63" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F64" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F65" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F66" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F67" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F68" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F69" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F70" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F71" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F72" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F73" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F74" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F75" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F76" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F77" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F78" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F79" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F80" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F81" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F82" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F83" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F84" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F85" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F86" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F87" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F88" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F89" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F90" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F91" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F92" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F93" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F94" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F95" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F96" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F97" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F98" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F99" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F100" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F101" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F102" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F103" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F104" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F105" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F106" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F107" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F108" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F109" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F110" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F111" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F112" r:id="rId108"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>